<commit_message>
Add Personal Investing Playbook dashboard and Excel download
</commit_message>
<xml_diff>
--- a/Personal_Investing_Playbook.xlsx
+++ b/Personal_Investing_Playbook.xlsx
@@ -8,19 +8,25 @@
   </bookViews>
   <sheets>
     <sheet name="Projection" sheetId="1" r:id="rId1"/>
-    <sheet name="Rebalance" sheetId="2" r:id="rId2"/>
+    <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="14">
   <si>
     <t>Month</t>
   </si>
   <si>
-    <t>Portfolio Value</t>
+    <t>Equity</t>
+  </si>
+  <si>
+    <t>Bond</t>
+  </si>
+  <si>
+    <t>Total Portfolio</t>
   </si>
   <si>
     <t>Total Invested</t>
@@ -32,14 +38,32 @@
     <t>Year</t>
   </si>
   <si>
-    <t>Rebalanced To 70/30</t>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Years</t>
+  </si>
+  <si>
+    <t>Total Invested (£)</t>
+  </si>
+  <si>
+    <t>Final Value (£)</t>
+  </si>
+  <si>
+    <t>Net Gain (£)</t>
+  </si>
+  <si>
+    <t>CAGR (%)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -55,13 +79,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F4E79"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -91,11 +129,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,7 +550,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Projection!$B$2:$B$121</c:f>
+              <c:f>Projection!$D$2:$D$121</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="120"/>
@@ -1259,7 +1298,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Projection!$C$2:$C$121</c:f>
+              <c:f>Projection!$E$2:$E$121</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="120"/>
@@ -1713,13 +1752,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
+      <xdr:col>14</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>76200</xdr:rowOff>
@@ -2029,10 +2068,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:G121"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2048,2044 +2087,2770 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
+        <v>350</v>
+      </c>
+      <c r="C2">
+        <v>150</v>
+      </c>
+      <c r="D2">
         <v>500</v>
       </c>
-      <c r="C2">
+      <c r="E2">
         <v>500</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>0</v>
       </c>
-      <c r="E2">
+      <c r="G2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
+        <v>682.736398247982</v>
+      </c>
+      <c r="C3">
+        <v>305.7729513933741</v>
+      </c>
+      <c r="D3">
         <v>988.5093496413562</v>
       </c>
-      <c r="C3">
+      <c r="E3">
         <v>1000</v>
       </c>
-      <c r="D3">
+      <c r="F3">
         <v>-11.49065035864385</v>
       </c>
-      <c r="E3">
+      <c r="G3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
+        <v>1049.911375545968</v>
+      </c>
+      <c r="C4">
+        <v>455.0930664521202</v>
+      </c>
+      <c r="D4">
         <v>1505.004441998088</v>
       </c>
-      <c r="C4">
+      <c r="E4">
         <v>1500</v>
       </c>
-      <c r="D4">
+      <c r="F4">
         <v>5.004441998087941</v>
       </c>
-      <c r="E4">
+      <c r="G4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
+        <v>1270.876140921829</v>
+      </c>
+      <c r="C5">
+        <v>611.0568688787981</v>
+      </c>
+      <c r="D5">
         <v>1881.933009800627</v>
       </c>
-      <c r="C5">
+      <c r="E5">
         <v>2000</v>
       </c>
-      <c r="D5">
+      <c r="F5">
         <v>-118.0669901993733</v>
       </c>
-      <c r="E5">
+      <c r="G5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
+        <v>1675.014090237908</v>
+      </c>
+      <c r="C6">
+        <v>772.9891341921283</v>
+      </c>
+      <c r="D6">
         <v>2448.003224430036</v>
       </c>
-      <c r="C6">
+      <c r="E6">
         <v>2500</v>
       </c>
-      <c r="D6">
+      <c r="F6">
         <v>-51.99677556996357</v>
       </c>
-      <c r="E6">
+      <c r="G6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
+        <v>2098.848658803168</v>
+      </c>
+      <c r="C7">
+        <v>917.6479682403982</v>
+      </c>
+      <c r="D7">
         <v>3016.496627043567</v>
       </c>
-      <c r="C7">
+      <c r="E7">
         <v>3000</v>
       </c>
-      <c r="D7">
+      <c r="F7">
         <v>16.4966270435666</v>
       </c>
-      <c r="E7">
+      <c r="G7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
+        <v>2428.017569608473</v>
+      </c>
+      <c r="C8">
+        <v>1022.636912979273</v>
+      </c>
+      <c r="D8">
         <v>3450.654482587746</v>
       </c>
-      <c r="C8">
+      <c r="E8">
         <v>3500</v>
       </c>
-      <c r="D8">
+      <c r="F8">
         <v>-49.34551741225414</v>
       </c>
-      <c r="E8">
+      <c r="G8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
+        <v>3132.28096634226</v>
+      </c>
+      <c r="C9">
+        <v>1170.737322191726</v>
+      </c>
+      <c r="D9">
         <v>4303.018288533986</v>
       </c>
-      <c r="C9">
+      <c r="E9">
         <v>4000</v>
       </c>
-      <c r="D9">
+      <c r="F9">
         <v>303.0182885339864</v>
       </c>
-      <c r="E9">
+      <c r="G9">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
+        <v>3754.233526931715</v>
+      </c>
+      <c r="C10">
+        <v>1340.422434171359</v>
+      </c>
+      <c r="D10">
         <v>5094.655961103073</v>
       </c>
-      <c r="C10">
+      <c r="E10">
         <v>4500</v>
       </c>
-      <c r="D10">
+      <c r="F10">
         <v>594.6559611030734</v>
       </c>
-      <c r="E10">
+      <c r="G10">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
+        <v>4103.86327162743</v>
+      </c>
+      <c r="C11">
+        <v>1758.798544983184</v>
+      </c>
+      <c r="D11">
         <v>5862.661816610615</v>
       </c>
-      <c r="C11">
+      <c r="E11">
         <v>5000</v>
       </c>
-      <c r="D11">
+      <c r="F11">
         <v>862.6618166106146</v>
       </c>
-      <c r="E11">
+      <c r="G11">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:7">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
+        <v>3995.003193581721</v>
+      </c>
+      <c r="C12">
+        <v>1887.30811768805</v>
+      </c>
+      <c r="D12">
         <v>5882.31131126977</v>
       </c>
-      <c r="C12">
+      <c r="E12">
         <v>5500</v>
       </c>
-      <c r="D12">
+      <c r="F12">
         <v>382.3113112697702</v>
       </c>
-      <c r="E12">
+      <c r="G12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:7">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
+        <v>4357.687161625511</v>
+      </c>
+      <c r="C13">
+        <v>1970.854555962956</v>
+      </c>
+      <c r="D13">
         <v>6328.541717588467</v>
       </c>
-      <c r="C13">
+      <c r="E13">
         <v>6000</v>
       </c>
-      <c r="D13">
+      <c r="F13">
         <v>328.5417175884668</v>
       </c>
-      <c r="E13">
+      <c r="G13">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:7">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
+        <v>4923.293038022603</v>
+      </c>
+      <c r="C14">
+        <v>2137.952865148623</v>
+      </c>
+      <c r="D14">
         <v>7061.245903171227</v>
       </c>
-      <c r="C14">
+      <c r="E14">
         <v>6500</v>
       </c>
-      <c r="D14">
+      <c r="F14">
         <v>561.2459031712269</v>
       </c>
-      <c r="E14">
+      <c r="G14">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:7">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
+        <v>5754.95922511416</v>
+      </c>
+      <c r="C15">
+        <v>2329.115964841303</v>
+      </c>
+      <c r="D15">
         <v>8084.075189955463</v>
       </c>
-      <c r="C15">
+      <c r="E15">
         <v>7000</v>
       </c>
-      <c r="D15">
+      <c r="F15">
         <v>1084.075189955463</v>
       </c>
-      <c r="E15">
+      <c r="G15">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:7">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16">
+        <v>6420.307241566103</v>
+      </c>
+      <c r="C16">
+        <v>2475.556370708431</v>
+      </c>
+      <c r="D16">
         <v>8895.863612274534</v>
       </c>
-      <c r="C16">
+      <c r="E16">
         <v>7500</v>
       </c>
-      <c r="D16">
+      <c r="F16">
         <v>1395.863612274534</v>
       </c>
-      <c r="E16">
+      <c r="G16">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:7">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17">
+        <v>7095.785186339706</v>
+      </c>
+      <c r="C17">
+        <v>2760.758726777236</v>
+      </c>
+      <c r="D17">
         <v>9856.543913116942</v>
       </c>
-      <c r="C17">
+      <c r="E17">
         <v>8000</v>
       </c>
-      <c r="D17">
+      <c r="F17">
         <v>1856.543913116942</v>
       </c>
-      <c r="E17">
+      <c r="G17">
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:7">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18">
+        <v>7509.550298228275</v>
+      </c>
+      <c r="C18">
+        <v>2841.426317805442</v>
+      </c>
+      <c r="D18">
         <v>10350.97661603372</v>
       </c>
-      <c r="C18">
+      <c r="E18">
         <v>8500</v>
       </c>
-      <c r="D18">
+      <c r="F18">
         <v>1850.976616033717</v>
       </c>
-      <c r="E18">
+      <c r="G18">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:7">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19">
+        <v>7423.58907578525</v>
+      </c>
+      <c r="C19">
+        <v>2893.656349538273</v>
+      </c>
+      <c r="D19">
         <v>10317.24542532352</v>
       </c>
-      <c r="C19">
+      <c r="E19">
         <v>9000</v>
       </c>
-      <c r="D19">
+      <c r="F19">
         <v>1317.245425323523</v>
       </c>
-      <c r="E19">
+      <c r="G19">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:7">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20">
+        <v>7720.379123321382</v>
+      </c>
+      <c r="C20">
+        <v>2898.78191292459</v>
+      </c>
+      <c r="D20">
         <v>10619.16103624597</v>
       </c>
-      <c r="C20">
+      <c r="E20">
         <v>9500</v>
       </c>
-      <c r="D20">
+      <c r="F20">
         <v>1119.161036245972</v>
       </c>
-      <c r="E20">
+      <c r="G20">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:7">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21">
+        <v>8938.610060262596</v>
+      </c>
+      <c r="C21">
+        <v>3094.106365146383</v>
+      </c>
+      <c r="D21">
         <v>12032.71642540898</v>
       </c>
-      <c r="C21">
+      <c r="E21">
         <v>10000</v>
       </c>
-      <c r="D21">
+      <c r="F21">
         <v>2032.716425408978</v>
       </c>
-      <c r="E21">
+      <c r="G21">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:7">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22">
+        <v>8805.934982162111</v>
+      </c>
+      <c r="C22">
+        <v>3251.994900936525</v>
+      </c>
+      <c r="D22">
         <v>12057.92988309864</v>
       </c>
-      <c r="C22">
+      <c r="E22">
         <v>10500</v>
       </c>
-      <c r="D22">
+      <c r="F22">
         <v>1557.929883098635</v>
       </c>
-      <c r="E22">
+      <c r="G22">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:7">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23">
+        <v>9294.53174830424</v>
+      </c>
+      <c r="C23">
+        <v>3386.746202625089</v>
+      </c>
+      <c r="D23">
         <v>12681.27795092933</v>
       </c>
-      <c r="C23">
+      <c r="E23">
         <v>11000</v>
       </c>
-      <c r="D23">
+      <c r="F23">
         <v>1681.277950929329</v>
       </c>
-      <c r="E23">
+      <c r="G23">
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:7">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24">
+        <v>10031.33503653914</v>
+      </c>
+      <c r="C24">
+        <v>4299.143587088201</v>
+      </c>
+      <c r="D24">
         <v>14330.47862362734</v>
       </c>
-      <c r="C24">
+      <c r="E24">
         <v>11500</v>
       </c>
-      <c r="D24">
+      <c r="F24">
         <v>2830.478623627339</v>
       </c>
-      <c r="E24">
+      <c r="G24">
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:7">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25">
+        <v>10791.43789933911</v>
+      </c>
+      <c r="C25">
+        <v>4590.788483169693</v>
+      </c>
+      <c r="D25">
         <v>15382.2263825088</v>
       </c>
-      <c r="C25">
+      <c r="E25">
         <v>12000</v>
       </c>
-      <c r="D25">
+      <c r="F25">
         <v>3382.226382508805</v>
       </c>
-      <c r="E25">
+      <c r="G25">
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:7">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26">
+        <v>10942.7811771113</v>
+      </c>
+      <c r="C26">
+        <v>4530.863214172809</v>
+      </c>
+      <c r="D26">
         <v>15473.64439128411</v>
       </c>
-      <c r="C26">
+      <c r="E26">
         <v>12500</v>
       </c>
-      <c r="D26">
+      <c r="F26">
         <v>2973.644391284113</v>
       </c>
-      <c r="E26">
+      <c r="G26">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:7">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27">
+        <v>11079.11452145562</v>
+      </c>
+      <c r="C27">
+        <v>4637.682870981317</v>
+      </c>
+      <c r="D27">
         <v>15716.79739243694</v>
       </c>
-      <c r="C27">
+      <c r="E27">
         <v>13000</v>
       </c>
-      <c r="D27">
+      <c r="F27">
         <v>2716.797392436936</v>
       </c>
-      <c r="E27">
+      <c r="G27">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:7">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28">
+        <v>12084.75224686684</v>
+      </c>
+      <c r="C28">
+        <v>4892.418142862055</v>
+      </c>
+      <c r="D28">
         <v>16977.17038972889</v>
       </c>
-      <c r="C28">
+      <c r="E28">
         <v>13500</v>
       </c>
-      <c r="D28">
+      <c r="F28">
         <v>3477.17038972889</v>
       </c>
-      <c r="E28">
+      <c r="G28">
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:7">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29">
+        <v>11479.42846281978</v>
+      </c>
+      <c r="C29">
+        <v>5143.636817549843</v>
+      </c>
+      <c r="D29">
         <v>16623.06528036962</v>
       </c>
-      <c r="C29">
+      <c r="E29">
         <v>14000</v>
       </c>
-      <c r="D29">
+      <c r="F29">
         <v>2623.065280369625</v>
       </c>
-      <c r="E29">
+      <c r="G29">
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:7">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30">
+        <v>12679.50495830802</v>
+      </c>
+      <c r="C30">
+        <v>5290.790502613574</v>
+      </c>
+      <c r="D30">
         <v>17970.2954609216</v>
       </c>
-      <c r="C30">
+      <c r="E30">
         <v>14500</v>
       </c>
-      <c r="D30">
+      <c r="F30">
         <v>3470.295460921596</v>
       </c>
-      <c r="E30">
+      <c r="G30">
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:7">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31">
+        <v>12740.90238244597</v>
+      </c>
+      <c r="C31">
+        <v>5578.629679894283</v>
+      </c>
+      <c r="D31">
         <v>18319.53206234026</v>
       </c>
-      <c r="C31">
+      <c r="E31">
         <v>15000</v>
       </c>
-      <c r="D31">
+      <c r="F31">
         <v>3319.532062340259</v>
       </c>
-      <c r="E31">
+      <c r="G31">
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:7">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32">
+        <v>13661.72697481586</v>
+      </c>
+      <c r="C32">
+        <v>5731.520398930203</v>
+      </c>
+      <c r="D32">
         <v>19393.24737374606</v>
       </c>
-      <c r="C32">
+      <c r="E32">
         <v>15500</v>
       </c>
-      <c r="D32">
+      <c r="F32">
         <v>3893.24737374606</v>
       </c>
-      <c r="E32">
+      <c r="G32">
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:7">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33">
+        <v>15341.09129995634</v>
+      </c>
+      <c r="C33">
+        <v>5754.435921790171</v>
+      </c>
+      <c r="D33">
         <v>21095.52722174651</v>
       </c>
-      <c r="C33">
+      <c r="E33">
         <v>16000</v>
       </c>
-      <c r="D33">
+      <c r="F33">
         <v>5095.52722174651</v>
       </c>
-      <c r="E33">
+      <c r="G33">
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:7">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34">
+        <v>14735.65349354881</v>
+      </c>
+      <c r="C34">
+        <v>6095.072743684185</v>
+      </c>
+      <c r="D34">
         <v>20830.72623723299</v>
       </c>
-      <c r="C34">
+      <c r="E34">
         <v>16500</v>
       </c>
-      <c r="D34">
+      <c r="F34">
         <v>4330.726237232993</v>
       </c>
-      <c r="E34">
+      <c r="G34">
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:7">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35">
+        <v>15228.22654025621</v>
+      </c>
+      <c r="C35">
+        <v>6423.10238201787</v>
+      </c>
+      <c r="D35">
         <v>21651.32892227408</v>
       </c>
-      <c r="C35">
+      <c r="E35">
         <v>17000</v>
       </c>
-      <c r="D35">
+      <c r="F35">
         <v>4651.328922274082</v>
       </c>
-      <c r="E35">
+      <c r="G35">
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:7">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36">
+        <v>15242.54265365152</v>
+      </c>
+      <c r="C36">
+        <v>6466.706075151546</v>
+      </c>
+      <c r="D36">
         <v>21709.24872880306</v>
       </c>
-      <c r="C36">
+      <c r="E36">
         <v>17500</v>
       </c>
-      <c r="D36">
+      <c r="F36">
         <v>4209.248728803064</v>
       </c>
-      <c r="E36">
+      <c r="G36">
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:7">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37">
+        <v>15191.85395533989</v>
+      </c>
+      <c r="C37">
+        <v>6879.251919965894</v>
+      </c>
+      <c r="D37">
         <v>22071.10587530578</v>
       </c>
-      <c r="C37">
+      <c r="E37">
         <v>18000</v>
       </c>
-      <c r="D37">
+      <c r="F37">
         <v>4071.105875305784</v>
       </c>
-      <c r="E37">
+      <c r="G37">
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:7">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38">
+        <v>15627.9051761333</v>
+      </c>
+      <c r="C38">
+        <v>7329.75983494951</v>
+      </c>
+      <c r="D38">
         <v>22957.6650110828</v>
       </c>
-      <c r="C38">
+      <c r="E38">
         <v>18500</v>
       </c>
-      <c r="D38">
+      <c r="F38">
         <v>4457.665011082805</v>
       </c>
-      <c r="E38">
+      <c r="G38">
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:7">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39">
+        <v>19342.57352784958</v>
+      </c>
+      <c r="C39">
+        <v>7771.209867054755</v>
+      </c>
+      <c r="D39">
         <v>27113.78339490433</v>
       </c>
-      <c r="C39">
+      <c r="E39">
         <v>19000</v>
       </c>
-      <c r="D39">
+      <c r="F39">
         <v>8113.783394904334</v>
       </c>
-      <c r="E39">
+      <c r="G39">
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:7">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40">
+        <v>19681.04430080857</v>
+      </c>
+      <c r="C40">
+        <v>7875.731586172455</v>
+      </c>
+      <c r="D40">
         <v>27556.77588698103</v>
       </c>
-      <c r="C40">
+      <c r="E40">
         <v>19500</v>
       </c>
-      <c r="D40">
+      <c r="F40">
         <v>8056.775886981028</v>
       </c>
-      <c r="E40">
+      <c r="G40">
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:7">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41">
+        <v>20076.73705183094</v>
+      </c>
+      <c r="C41">
+        <v>7631.212317084874</v>
+      </c>
+      <c r="D41">
         <v>27707.94936891581</v>
       </c>
-      <c r="C41">
+      <c r="E41">
         <v>20000</v>
       </c>
-      <c r="D41">
+      <c r="F41">
         <v>7707.949368915812</v>
       </c>
-      <c r="E41">
+      <c r="G41">
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:7">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42">
+        <v>20885.18353303957</v>
+      </c>
+      <c r="C42">
+        <v>7881.719218899137</v>
+      </c>
+      <c r="D42">
         <v>28766.90275193871</v>
       </c>
-      <c r="C42">
+      <c r="E42">
         <v>20500</v>
       </c>
-      <c r="D42">
+      <c r="F42">
         <v>8266.902751938705</v>
       </c>
-      <c r="E42">
+      <c r="G42">
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:7">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43">
+        <v>18891.29928177795</v>
+      </c>
+      <c r="C43">
+        <v>7874.471617368506</v>
+      </c>
+      <c r="D43">
         <v>26765.77089914646</v>
       </c>
-      <c r="C43">
+      <c r="E43">
         <v>21000</v>
       </c>
-      <c r="D43">
+      <c r="F43">
         <v>5765.770899146461</v>
       </c>
-      <c r="E43">
+      <c r="G43">
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:7">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44">
+        <v>20600.5806601143</v>
+      </c>
+      <c r="C44">
+        <v>7978.961158461967</v>
+      </c>
+      <c r="D44">
         <v>28579.54181857626</v>
       </c>
-      <c r="C44">
+      <c r="E44">
         <v>21500</v>
       </c>
-      <c r="D44">
+      <c r="F44">
         <v>7079.541818576265</v>
       </c>
-      <c r="E44">
+      <c r="G44">
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:7">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45">
+        <v>19538.16830090457</v>
+      </c>
+      <c r="C45">
+        <v>8173.700482034423</v>
+      </c>
+      <c r="D45">
         <v>27711.868782939</v>
       </c>
-      <c r="C45">
+      <c r="E45">
         <v>22000</v>
       </c>
-      <c r="D45">
+      <c r="F45">
         <v>5711.868782938996</v>
       </c>
-      <c r="E45">
+      <c r="G45">
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:7">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46">
+        <v>20816.49106489516</v>
+      </c>
+      <c r="C46">
+        <v>8480.002355525012</v>
+      </c>
+      <c r="D46">
         <v>29296.49342042017</v>
       </c>
-      <c r="C46">
+      <c r="E46">
         <v>22500</v>
       </c>
-      <c r="D46">
+      <c r="F46">
         <v>6796.493420420167</v>
       </c>
-      <c r="E46">
+      <c r="G46">
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:7">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47">
+        <v>21085.72874621846</v>
+      </c>
+      <c r="C47">
+        <v>8861.330297651381</v>
+      </c>
+      <c r="D47">
         <v>29947.05904386984</v>
       </c>
-      <c r="C47">
+      <c r="E47">
         <v>23000</v>
       </c>
-      <c r="D47">
+      <c r="F47">
         <v>6947.059043869842</v>
       </c>
-      <c r="E47">
+      <c r="G47">
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:7">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48">
+        <v>22764.90939347252</v>
+      </c>
+      <c r="C48">
+        <v>8994.842220992608</v>
+      </c>
+      <c r="D48">
         <v>31759.75161446513</v>
       </c>
-      <c r="C48">
+      <c r="E48">
         <v>23500</v>
       </c>
-      <c r="D48">
+      <c r="F48">
         <v>8259.751614465131</v>
       </c>
-      <c r="E48">
+      <c r="G48">
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:5">
+    <row r="49" spans="1:7">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49">
+        <v>24031.9514910508</v>
+      </c>
+      <c r="C49">
+        <v>8843.840347684916</v>
+      </c>
+      <c r="D49">
         <v>32875.79183873572</v>
       </c>
-      <c r="C49">
+      <c r="E49">
         <v>24000</v>
       </c>
-      <c r="D49">
+      <c r="F49">
         <v>8875.79183873572</v>
       </c>
-      <c r="E49">
+      <c r="G49">
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:5">
+    <row r="50" spans="1:7">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50">
+        <v>23936.52874906003</v>
+      </c>
+      <c r="C50">
+        <v>9060.663963767372</v>
+      </c>
+      <c r="D50">
         <v>32997.1927128274</v>
       </c>
-      <c r="C50">
+      <c r="E50">
         <v>24500</v>
       </c>
-      <c r="D50">
+      <c r="F50">
         <v>8497.192712827396</v>
       </c>
-      <c r="E50">
+      <c r="G50">
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:5">
+    <row r="51" spans="1:7">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51">
+        <v>24427.26258350546</v>
+      </c>
+      <c r="C51">
+        <v>9177.383656304422</v>
+      </c>
+      <c r="D51">
         <v>33604.64623980988</v>
       </c>
-      <c r="C51">
+      <c r="E51">
         <v>25000</v>
       </c>
-      <c r="D51">
+      <c r="F51">
         <v>8604.646239809881</v>
       </c>
-      <c r="E51">
+      <c r="G51">
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:5">
+    <row r="52" spans="1:7">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52">
+        <v>27725.38667752486</v>
+      </c>
+      <c r="C52">
+        <v>9327.301667454472</v>
+      </c>
+      <c r="D52">
         <v>37052.68834497933</v>
       </c>
-      <c r="C52">
+      <c r="E52">
         <v>25500</v>
       </c>
-      <c r="D52">
+      <c r="F52">
         <v>11552.68834497933</v>
       </c>
-      <c r="E52">
+      <c r="G52">
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
+    <row r="53" spans="1:7">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53">
+        <v>26859.00671800763</v>
+      </c>
+      <c r="C53">
+        <v>11511.00287914613</v>
+      </c>
+      <c r="D53">
         <v>38370.00959715376</v>
       </c>
-      <c r="C53">
+      <c r="E53">
         <v>26000</v>
       </c>
-      <c r="D53">
+      <c r="F53">
         <v>12370.00959715376</v>
       </c>
-      <c r="E53">
+      <c r="G53">
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:5">
+    <row r="54" spans="1:7">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54">
+        <v>27693.51437720398</v>
+      </c>
+      <c r="C54">
+        <v>11822.7171326567</v>
+      </c>
+      <c r="D54">
         <v>39516.23150986069</v>
       </c>
-      <c r="C54">
+      <c r="E54">
         <v>26500</v>
       </c>
-      <c r="D54">
+      <c r="F54">
         <v>13016.23150986069</v>
       </c>
-      <c r="E54">
+      <c r="G54">
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:5">
+    <row r="55" spans="1:7">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55">
+        <v>23987.08315734437</v>
+      </c>
+      <c r="C55">
+        <v>11922.31510942734</v>
+      </c>
+      <c r="D55">
         <v>35909.39826677171</v>
       </c>
-      <c r="C55">
+      <c r="E55">
         <v>27000</v>
       </c>
-      <c r="D55">
+      <c r="F55">
         <v>8909.398266771714</v>
       </c>
-      <c r="E55">
+      <c r="G55">
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:5">
+    <row r="56" spans="1:7">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56">
+        <v>23982.7487493481</v>
+      </c>
+      <c r="C56">
+        <v>12060.4297877827</v>
+      </c>
+      <c r="D56">
         <v>36043.1785371308</v>
       </c>
-      <c r="C56">
+      <c r="E56">
         <v>27500</v>
       </c>
-      <c r="D56">
+      <c r="F56">
         <v>8543.1785371308</v>
       </c>
-      <c r="E56">
+      <c r="G56">
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:5">
+    <row r="57" spans="1:7">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57">
+        <v>28181.4701858008</v>
+      </c>
+      <c r="C57">
+        <v>12371.2652585699</v>
+      </c>
+      <c r="D57">
         <v>40552.73544437071</v>
       </c>
-      <c r="C57">
+      <c r="E57">
         <v>28000</v>
       </c>
-      <c r="D57">
+      <c r="F57">
         <v>12552.73544437071</v>
       </c>
-      <c r="E57">
+      <c r="G57">
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:5">
+    <row r="58" spans="1:7">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58">
+        <v>28423.54400944476</v>
+      </c>
+      <c r="C58">
+        <v>13345.61865462945</v>
+      </c>
+      <c r="D58">
         <v>41769.16266407421</v>
       </c>
-      <c r="C58">
+      <c r="E58">
         <v>28500</v>
       </c>
-      <c r="D58">
+      <c r="F58">
         <v>13269.16266407421</v>
       </c>
-      <c r="E58">
+      <c r="G58">
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:5">
+    <row r="59" spans="1:7">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59">
+        <v>29363.1280359337</v>
+      </c>
+      <c r="C59">
+        <v>13649.78048551211</v>
+      </c>
+      <c r="D59">
         <v>43012.9085214458</v>
       </c>
-      <c r="C59">
+      <c r="E59">
         <v>29000</v>
       </c>
-      <c r="D59">
+      <c r="F59">
         <v>14012.9085214458</v>
       </c>
-      <c r="E59">
+      <c r="G59">
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:5">
+    <row r="60" spans="1:7">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60">
+        <v>30033.54653727927</v>
+      </c>
+      <c r="C60">
+        <v>13419.0666932052</v>
+      </c>
+      <c r="D60">
         <v>43452.61323048447</v>
       </c>
-      <c r="C60">
+      <c r="E60">
         <v>29500</v>
       </c>
-      <c r="D60">
+      <c r="F60">
         <v>13952.61323048447</v>
       </c>
-      <c r="E60">
+      <c r="G60">
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:5">
+    <row r="61" spans="1:7">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61">
+        <v>27749.2663591324</v>
+      </c>
+      <c r="C61">
+        <v>13774.66001629046</v>
+      </c>
+      <c r="D61">
         <v>41523.92637542286</v>
       </c>
-      <c r="C61">
+      <c r="E61">
         <v>30000</v>
       </c>
-      <c r="D61">
+      <c r="F61">
         <v>11523.92637542286</v>
       </c>
-      <c r="E61">
+      <c r="G61">
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:5">
+    <row r="62" spans="1:7">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62">
+        <v>26541.8806071267</v>
+      </c>
+      <c r="C62">
+        <v>13565.63220879967</v>
+      </c>
+      <c r="D62">
         <v>40107.51281592637</v>
       </c>
-      <c r="C62">
+      <c r="E62">
         <v>30500</v>
       </c>
-      <c r="D62">
+      <c r="F62">
         <v>9607.51281592637</v>
       </c>
-      <c r="E62">
+      <c r="G62">
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:5">
+    <row r="63" spans="1:7">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63">
+        <v>26079.77331777482</v>
+      </c>
+      <c r="C63">
+        <v>11177.04570761778</v>
+      </c>
+      <c r="D63">
         <v>37256.8190253926</v>
       </c>
-      <c r="C63">
+      <c r="E63">
         <v>31000</v>
       </c>
-      <c r="D63">
+      <c r="F63">
         <v>6256.8190253926</v>
       </c>
-      <c r="E63">
+      <c r="G63">
         <v>6</v>
       </c>
     </row>
-    <row r="64" spans="1:5">
+    <row r="64" spans="1:7">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64">
+        <v>25237.22819350819</v>
+      </c>
+      <c r="C64">
+        <v>11956.62038258733</v>
+      </c>
+      <c r="D64">
         <v>37193.84857609552</v>
       </c>
-      <c r="C64">
+      <c r="E64">
         <v>31500</v>
       </c>
-      <c r="D64">
+      <c r="F64">
         <v>5693.848576095515</v>
       </c>
-      <c r="E64">
+      <c r="G64">
         <v>6</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:7">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65">
+        <v>27776.45240735729</v>
+      </c>
+      <c r="C65">
+        <v>12030.39104944256</v>
+      </c>
+      <c r="D65">
         <v>39806.84345679985</v>
       </c>
-      <c r="C65">
+      <c r="E65">
         <v>32000</v>
       </c>
-      <c r="D65">
+      <c r="F65">
         <v>7806.843456799848</v>
       </c>
-      <c r="E65">
+      <c r="G65">
         <v>6</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:7">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66">
+        <v>28092.77966770863</v>
+      </c>
+      <c r="C66">
+        <v>12044.6690136359</v>
+      </c>
+      <c r="D66">
         <v>40137.44868134454</v>
       </c>
-      <c r="C66">
+      <c r="E66">
         <v>32500</v>
       </c>
-      <c r="D66">
+      <c r="F66">
         <v>7637.44868134454</v>
       </c>
-      <c r="E66">
+      <c r="G66">
         <v>6</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:7">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67">
+        <v>32112.67907663783</v>
+      </c>
+      <c r="C67">
+        <v>12358.63628654142</v>
+      </c>
+      <c r="D67">
         <v>44471.31536317925</v>
       </c>
-      <c r="C67">
+      <c r="E67">
         <v>33000</v>
       </c>
-      <c r="D67">
+      <c r="F67">
         <v>11471.31536317925</v>
       </c>
-      <c r="E67">
+      <c r="G67">
         <v>6</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:7">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68">
+        <v>35368.79034741985</v>
+      </c>
+      <c r="C68">
+        <v>12771.67493478082</v>
+      </c>
+      <c r="D68">
         <v>48140.46528220066</v>
       </c>
-      <c r="C68">
+      <c r="E68">
         <v>33500</v>
       </c>
-      <c r="D68">
+      <c r="F68">
         <v>14640.46528220066</v>
       </c>
-      <c r="E68">
+      <c r="G68">
         <v>6</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:7">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69">
+        <v>38438.07452912757</v>
+      </c>
+      <c r="C69">
+        <v>13542.47651227506</v>
+      </c>
+      <c r="D69">
         <v>51980.55104140262</v>
       </c>
-      <c r="C69">
+      <c r="E69">
         <v>34000</v>
       </c>
-      <c r="D69">
+      <c r="F69">
         <v>17980.55104140262</v>
       </c>
-      <c r="E69">
+      <c r="G69">
         <v>6</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:7">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70">
+        <v>38596.61185006891</v>
+      </c>
+      <c r="C70">
+        <v>16541.40507860096</v>
+      </c>
+      <c r="D70">
         <v>55138.01692866987</v>
       </c>
-      <c r="C70">
+      <c r="E70">
         <v>34500</v>
       </c>
-      <c r="D70">
+      <c r="F70">
         <v>20638.01692866987</v>
       </c>
-      <c r="E70">
+      <c r="G70">
         <v>6</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:7">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71">
+        <v>36734.74360208779</v>
+      </c>
+      <c r="C71">
+        <v>16118.7930297608</v>
+      </c>
+      <c r="D71">
         <v>52853.5366318486</v>
       </c>
-      <c r="C71">
+      <c r="E71">
         <v>35000</v>
       </c>
-      <c r="D71">
+      <c r="F71">
         <v>17853.5366318486</v>
       </c>
-      <c r="E71">
+      <c r="G71">
         <v>6</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:7">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72">
+        <v>36532.04918036499</v>
+      </c>
+      <c r="C72">
+        <v>16838.73471713764</v>
+      </c>
+      <c r="D72">
         <v>53370.78389750262</v>
       </c>
-      <c r="C72">
+      <c r="E72">
         <v>35500</v>
       </c>
-      <c r="D72">
+      <c r="F72">
         <v>17870.78389750262</v>
       </c>
-      <c r="E72">
+      <c r="G72">
         <v>6</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:7">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73">
+        <v>41813.37242263566</v>
+      </c>
+      <c r="C73">
+        <v>17274.88962281866</v>
+      </c>
+      <c r="D73">
         <v>59088.26204545432</v>
       </c>
-      <c r="C73">
+      <c r="E73">
         <v>36000</v>
       </c>
-      <c r="D73">
+      <c r="F73">
         <v>23088.26204545432</v>
       </c>
-      <c r="E73">
+      <c r="G73">
         <v>6</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:7">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74">
+        <v>41467.93398066994</v>
+      </c>
+      <c r="C74">
+        <v>17794.73213083777</v>
+      </c>
+      <c r="D74">
         <v>59262.6661115077</v>
       </c>
-      <c r="C74">
+      <c r="E74">
         <v>36500</v>
       </c>
-      <c r="D74">
+      <c r="F74">
         <v>22762.6661115077</v>
       </c>
-      <c r="E74">
+      <c r="G74">
         <v>7</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:7">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75">
+        <v>46299.45494159935</v>
+      </c>
+      <c r="C75">
+        <v>17506.24614085012</v>
+      </c>
+      <c r="D75">
         <v>63805.70108244946</v>
       </c>
-      <c r="C75">
+      <c r="E75">
         <v>37000</v>
       </c>
-      <c r="D75">
+      <c r="F75">
         <v>26805.70108244946</v>
       </c>
-      <c r="E75">
+      <c r="G75">
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:7">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76">
+        <v>44945.68204356143</v>
+      </c>
+      <c r="C76">
+        <v>17781.23608635828</v>
+      </c>
+      <c r="D76">
         <v>62726.91812991971</v>
       </c>
-      <c r="C76">
+      <c r="E76">
         <v>37500</v>
       </c>
-      <c r="D76">
+      <c r="F76">
         <v>25226.91812991971</v>
       </c>
-      <c r="E76">
+      <c r="G76">
         <v>7</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:7">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77">
+        <v>44620.36396848682</v>
+      </c>
+      <c r="C77">
+        <v>18110.22235877745</v>
+      </c>
+      <c r="D77">
         <v>62730.58632726426</v>
       </c>
-      <c r="C77">
+      <c r="E77">
         <v>38000</v>
       </c>
-      <c r="D77">
+      <c r="F77">
         <v>24730.58632726426</v>
       </c>
-      <c r="E77">
+      <c r="G77">
         <v>7</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:7">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78">
+        <v>47655.11529546415</v>
+      </c>
+      <c r="C78">
+        <v>18489.63439822188</v>
+      </c>
+      <c r="D78">
         <v>66144.74969368603</v>
       </c>
-      <c r="C78">
+      <c r="E78">
         <v>38500</v>
       </c>
-      <c r="D78">
+      <c r="F78">
         <v>27644.74969368603</v>
       </c>
-      <c r="E78">
+      <c r="G78">
         <v>7</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:7">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79">
+        <v>47224.32291756652</v>
+      </c>
+      <c r="C79">
+        <v>18307.46150906686</v>
+      </c>
+      <c r="D79">
         <v>65531.78442663337</v>
       </c>
-      <c r="C79">
+      <c r="E79">
         <v>39000</v>
       </c>
-      <c r="D79">
+      <c r="F79">
         <v>26531.78442663337</v>
       </c>
-      <c r="E79">
+      <c r="G79">
         <v>7</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:7">
       <c r="A80">
         <v>79</v>
       </c>
       <c r="B80">
+        <v>40707.16365439421</v>
+      </c>
+      <c r="C80">
+        <v>18525.10881774692</v>
+      </c>
+      <c r="D80">
         <v>59232.27247214113</v>
       </c>
-      <c r="C80">
+      <c r="E80">
         <v>39500</v>
       </c>
-      <c r="D80">
+      <c r="F80">
         <v>19732.27247214113</v>
       </c>
-      <c r="E80">
+      <c r="G80">
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
+    <row r="81" spans="1:7">
       <c r="A81">
         <v>80</v>
       </c>
       <c r="B81">
+        <v>45149.59385975154</v>
+      </c>
+      <c r="C81">
+        <v>19172.49939813386</v>
+      </c>
+      <c r="D81">
         <v>64322.0932578854</v>
       </c>
-      <c r="C81">
+      <c r="E81">
         <v>40000</v>
       </c>
-      <c r="D81">
+      <c r="F81">
         <v>24322.0932578854</v>
       </c>
-      <c r="E81">
+      <c r="G81">
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:5">
+    <row r="82" spans="1:7">
       <c r="A82">
         <v>81</v>
       </c>
       <c r="B82">
+        <v>49239.1309771755</v>
+      </c>
+      <c r="C82">
+        <v>19877.84248778461</v>
+      </c>
+      <c r="D82">
         <v>69116.9734649601</v>
       </c>
-      <c r="C82">
+      <c r="E82">
         <v>40500</v>
       </c>
-      <c r="D82">
+      <c r="F82">
         <v>28616.9734649601</v>
       </c>
-      <c r="E82">
+      <c r="G82">
         <v>7</v>
       </c>
     </row>
-    <row r="83" spans="1:5">
+    <row r="83" spans="1:7">
       <c r="A83">
         <v>82</v>
       </c>
       <c r="B83">
+        <v>45358.94876378917</v>
+      </c>
+      <c r="C83">
+        <v>19512.00320372995</v>
+      </c>
+      <c r="D83">
         <v>64870.95196751913</v>
       </c>
-      <c r="C83">
+      <c r="E83">
         <v>41000</v>
       </c>
-      <c r="D83">
+      <c r="F83">
         <v>23870.95196751913</v>
       </c>
-      <c r="E83">
+      <c r="G83">
         <v>7</v>
       </c>
     </row>
-    <row r="84" spans="1:5">
+    <row r="84" spans="1:7">
       <c r="A84">
         <v>83</v>
       </c>
       <c r="B84">
+        <v>42416.29308105358</v>
+      </c>
+      <c r="C84">
+        <v>19808.71556211488</v>
+      </c>
+      <c r="D84">
         <v>62225.00864316847</v>
       </c>
-      <c r="C84">
+      <c r="E84">
         <v>41500</v>
       </c>
-      <c r="D84">
+      <c r="F84">
         <v>20725.00864316847</v>
       </c>
-      <c r="E84">
+      <c r="G84">
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:5">
+    <row r="85" spans="1:7">
       <c r="A85">
         <v>84</v>
       </c>
       <c r="B85">
+        <v>40047.26283366074</v>
+      </c>
+      <c r="C85">
+        <v>20894.18179359982</v>
+      </c>
+      <c r="D85">
         <v>60941.44462726057</v>
       </c>
-      <c r="C85">
+      <c r="E85">
         <v>42000</v>
       </c>
-      <c r="D85">
+      <c r="F85">
         <v>18941.44462726057</v>
       </c>
-      <c r="E85">
+      <c r="G85">
         <v>7</v>
       </c>
     </row>
-    <row r="86" spans="1:5">
+    <row r="86" spans="1:7">
       <c r="A86">
         <v>85</v>
       </c>
       <c r="B86">
+        <v>41481.58081218816</v>
+      </c>
+      <c r="C86">
+        <v>20714.86976582387</v>
+      </c>
+      <c r="D86">
         <v>62196.45057801202</v>
       </c>
-      <c r="C86">
+      <c r="E86">
         <v>42500</v>
       </c>
-      <c r="D86">
+      <c r="F86">
         <v>19696.45057801202</v>
       </c>
-      <c r="E86">
+      <c r="G86">
         <v>8</v>
       </c>
     </row>
-    <row r="87" spans="1:5">
+    <row r="87" spans="1:7">
       <c r="A87">
         <v>86</v>
       </c>
       <c r="B87">
+        <v>45112.51849183347</v>
+      </c>
+      <c r="C87">
+        <v>20584.89449181911</v>
+      </c>
+      <c r="D87">
         <v>65697.41298365258</v>
       </c>
-      <c r="C87">
+      <c r="E87">
         <v>43000</v>
       </c>
-      <c r="D87">
+      <c r="F87">
         <v>22697.41298365258</v>
       </c>
-      <c r="E87">
+      <c r="G87">
         <v>8</v>
       </c>
     </row>
-    <row r="88" spans="1:5">
+    <row r="88" spans="1:7">
       <c r="A88">
         <v>87</v>
       </c>
       <c r="B88">
+        <v>45975.85974193074</v>
+      </c>
+      <c r="C88">
+        <v>20979.76999699036</v>
+      </c>
+      <c r="D88">
         <v>66955.6297389211</v>
       </c>
-      <c r="C88">
+      <c r="E88">
         <v>43500</v>
       </c>
-      <c r="D88">
+      <c r="F88">
         <v>23455.6297389211</v>
       </c>
-      <c r="E88">
+      <c r="G88">
         <v>8</v>
       </c>
     </row>
-    <row r="89" spans="1:5">
+    <row r="89" spans="1:7">
       <c r="A89">
         <v>88</v>
       </c>
       <c r="B89">
+        <v>45494.8575825285</v>
+      </c>
+      <c r="C89">
+        <v>21601.72986006184</v>
+      </c>
+      <c r="D89">
         <v>67096.58744259035</v>
       </c>
-      <c r="C89">
+      <c r="E89">
         <v>44000</v>
       </c>
-      <c r="D89">
+      <c r="F89">
         <v>23096.58744259035</v>
       </c>
-      <c r="E89">
+      <c r="G89">
         <v>8</v>
       </c>
     </row>
-    <row r="90" spans="1:5">
+    <row r="90" spans="1:7">
       <c r="A90">
         <v>89</v>
       </c>
       <c r="B90">
+        <v>45933.44781792784</v>
+      </c>
+      <c r="C90">
+        <v>22626.18021637875</v>
+      </c>
+      <c r="D90">
         <v>68559.6280343066</v>
       </c>
-      <c r="C90">
+      <c r="E90">
         <v>44500</v>
       </c>
-      <c r="D90">
+      <c r="F90">
         <v>24059.6280343066</v>
       </c>
-      <c r="E90">
+      <c r="G90">
         <v>8</v>
       </c>
     </row>
-    <row r="91" spans="1:5">
+    <row r="91" spans="1:7">
       <c r="A91">
         <v>90</v>
       </c>
       <c r="B91">
+        <v>47286.83764691513</v>
+      </c>
+      <c r="C91">
+        <v>24480.24970805406</v>
+      </c>
+      <c r="D91">
         <v>71767.08735496919</v>
       </c>
-      <c r="C91">
+      <c r="E91">
         <v>45000</v>
       </c>
-      <c r="D91">
+      <c r="F91">
         <v>26767.08735496919</v>
       </c>
-      <c r="E91">
+      <c r="G91">
         <v>8</v>
       </c>
     </row>
-    <row r="92" spans="1:5">
+    <row r="92" spans="1:7">
       <c r="A92">
         <v>91</v>
       </c>
       <c r="B92">
+        <v>45608.12753596817</v>
+      </c>
+      <c r="C92">
+        <v>24049.99150861985</v>
+      </c>
+      <c r="D92">
         <v>69658.11904458801</v>
       </c>
-      <c r="C92">
+      <c r="E92">
         <v>45500</v>
       </c>
-      <c r="D92">
+      <c r="F92">
         <v>24158.11904458801</v>
       </c>
-      <c r="E92">
+      <c r="G92">
         <v>8</v>
       </c>
     </row>
-    <row r="93" spans="1:5">
+    <row r="93" spans="1:7">
       <c r="A93">
         <v>92</v>
       </c>
       <c r="B93">
+        <v>50116.31016142028</v>
+      </c>
+      <c r="C93">
+        <v>24718.69962239381</v>
+      </c>
+      <c r="D93">
         <v>74835.00978381408</v>
       </c>
-      <c r="C93">
+      <c r="E93">
         <v>46000</v>
       </c>
-      <c r="D93">
+      <c r="F93">
         <v>28835.00978381408</v>
       </c>
-      <c r="E93">
+      <c r="G93">
         <v>8</v>
       </c>
     </row>
-    <row r="94" spans="1:5">
+    <row r="94" spans="1:7">
       <c r="A94">
         <v>93</v>
       </c>
       <c r="B94">
+        <v>51591.08020784615</v>
+      </c>
+      <c r="C94">
+        <v>25425.80669708026</v>
+      </c>
+      <c r="D94">
         <v>77016.88690492642</v>
       </c>
-      <c r="C94">
+      <c r="E94">
         <v>46500</v>
       </c>
-      <c r="D94">
+      <c r="F94">
         <v>30516.88690492642</v>
       </c>
-      <c r="E94">
+      <c r="G94">
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="1:5">
+    <row r="95" spans="1:7">
       <c r="A95">
         <v>94</v>
       </c>
       <c r="B95">
+        <v>50282.28437901417</v>
+      </c>
+      <c r="C95">
+        <v>25518.58242285543</v>
+      </c>
+      <c r="D95">
         <v>75800.8668018696</v>
       </c>
-      <c r="C95">
+      <c r="E95">
         <v>47000</v>
       </c>
-      <c r="D95">
+      <c r="F95">
         <v>28800.8668018696</v>
       </c>
-      <c r="E95">
+      <c r="G95">
         <v>8</v>
       </c>
     </row>
-    <row r="96" spans="1:5">
+    <row r="96" spans="1:7">
       <c r="A96">
         <v>95</v>
       </c>
       <c r="B96">
+        <v>54504.87433180366</v>
+      </c>
+      <c r="C96">
+        <v>24850.05716215073</v>
+      </c>
+      <c r="D96">
         <v>79354.93149395438</v>
       </c>
-      <c r="C96">
+      <c r="E96">
         <v>47500</v>
       </c>
-      <c r="D96">
+      <c r="F96">
         <v>31854.93149395438</v>
       </c>
-      <c r="E96">
+      <c r="G96">
         <v>8</v>
       </c>
     </row>
-    <row r="97" spans="1:5">
+    <row r="97" spans="1:7">
       <c r="A97">
         <v>96</v>
       </c>
       <c r="B97">
+        <v>57042.49396730401</v>
+      </c>
+      <c r="C97">
+        <v>25686.0854834202</v>
+      </c>
+      <c r="D97">
         <v>82728.57945072421</v>
       </c>
-      <c r="C97">
+      <c r="E97">
         <v>48000</v>
       </c>
-      <c r="D97">
+      <c r="F97">
         <v>34728.57945072421</v>
       </c>
-      <c r="E97">
+      <c r="G97">
         <v>8</v>
       </c>
     </row>
-    <row r="98" spans="1:5">
+    <row r="98" spans="1:7">
       <c r="A98">
         <v>97</v>
       </c>
       <c r="B98">
+        <v>56880.06583590477</v>
+      </c>
+      <c r="C98">
+        <v>25029.42982065315</v>
+      </c>
+      <c r="D98">
         <v>81909.49565655791</v>
       </c>
-      <c r="C98">
+      <c r="E98">
         <v>48500</v>
       </c>
-      <c r="D98">
+      <c r="F98">
         <v>33409.49565655791</v>
       </c>
-      <c r="E98">
+      <c r="G98">
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:5">
+    <row r="99" spans="1:7">
       <c r="A99">
         <v>98</v>
       </c>
       <c r="B99">
+        <v>56725.4168257611</v>
+      </c>
+      <c r="C99">
+        <v>25468.47782696574</v>
+      </c>
+      <c r="D99">
         <v>82193.89465272684</v>
       </c>
-      <c r="C99">
+      <c r="E99">
         <v>49000</v>
       </c>
-      <c r="D99">
+      <c r="F99">
         <v>33193.89465272684</v>
       </c>
-      <c r="E99">
+      <c r="G99">
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:5">
+    <row r="100" spans="1:7">
       <c r="A100">
         <v>99</v>
       </c>
       <c r="B100">
+        <v>61428.79273175882</v>
+      </c>
+      <c r="C100">
+        <v>25919.92859990087</v>
+      </c>
+      <c r="D100">
         <v>87348.72133165969</v>
       </c>
-      <c r="C100">
+      <c r="E100">
         <v>49500</v>
       </c>
-      <c r="D100">
+      <c r="F100">
         <v>37848.72133165969</v>
       </c>
-      <c r="E100">
+      <c r="G100">
         <v>9</v>
       </c>
     </row>
-    <row r="101" spans="1:5">
+    <row r="101" spans="1:7">
       <c r="A101">
         <v>100</v>
       </c>
       <c r="B101">
+        <v>61986.14884633867</v>
+      </c>
+      <c r="C101">
+        <v>25349.9555592131</v>
+      </c>
+      <c r="D101">
         <v>87336.10440555177</v>
       </c>
-      <c r="C101">
+      <c r="E101">
         <v>50000</v>
       </c>
-      <c r="D101">
+      <c r="F101">
         <v>37336.10440555177</v>
       </c>
-      <c r="E101">
+      <c r="G101">
         <v>9</v>
       </c>
     </row>
-    <row r="102" spans="1:5">
+    <row r="102" spans="1:7">
       <c r="A102">
         <v>101</v>
       </c>
       <c r="B102">
+        <v>60843.00230716605</v>
+      </c>
+      <c r="C102">
+        <v>25881.05076925156</v>
+      </c>
+      <c r="D102">
         <v>86724.05307641761</v>
       </c>
-      <c r="C102">
+      <c r="E102">
         <v>50500</v>
       </c>
-      <c r="D102">
+      <c r="F102">
         <v>36224.05307641761</v>
       </c>
-      <c r="E102">
+      <c r="G102">
         <v>9</v>
       </c>
     </row>
-    <row r="103" spans="1:5">
+    <row r="103" spans="1:7">
       <c r="A103">
         <v>102</v>
       </c>
       <c r="B103">
+        <v>56113.52296255182</v>
+      </c>
+      <c r="C103">
+        <v>26641.43368909832</v>
+      </c>
+      <c r="D103">
         <v>82754.95665165014</v>
       </c>
-      <c r="C103">
+      <c r="E103">
         <v>51000</v>
       </c>
-      <c r="D103">
+      <c r="F103">
         <v>31754.95665165014</v>
       </c>
-      <c r="E103">
+      <c r="G103">
         <v>9</v>
       </c>
     </row>
-    <row r="104" spans="1:5">
+    <row r="104" spans="1:7">
       <c r="A104">
         <v>103</v>
       </c>
       <c r="B104">
+        <v>63122.08348885821</v>
+      </c>
+      <c r="C104">
+        <v>26424.39222528648</v>
+      </c>
+      <c r="D104">
         <v>89546.47571414469</v>
       </c>
-      <c r="C104">
+      <c r="E104">
         <v>51500</v>
       </c>
-      <c r="D104">
+      <c r="F104">
         <v>38046.47571414469</v>
       </c>
-      <c r="E104">
+      <c r="G104">
         <v>9</v>
       </c>
     </row>
-    <row r="105" spans="1:5">
+    <row r="105" spans="1:7">
       <c r="A105">
         <v>104</v>
       </c>
       <c r="B105">
+        <v>61157.65367150508</v>
+      </c>
+      <c r="C105">
+        <v>26914.15347885093</v>
+      </c>
+      <c r="D105">
         <v>88071.80715035601</v>
       </c>
-      <c r="C105">
+      <c r="E105">
         <v>52000</v>
       </c>
-      <c r="D105">
+      <c r="F105">
         <v>36071.80715035601</v>
       </c>
-      <c r="E105">
+      <c r="G105">
         <v>9</v>
       </c>
     </row>
-    <row r="106" spans="1:5">
+    <row r="106" spans="1:7">
       <c r="A106">
         <v>105</v>
       </c>
       <c r="B106">
+        <v>58866.415602185</v>
+      </c>
+      <c r="C106">
+        <v>29763.19302779956</v>
+      </c>
+      <c r="D106">
         <v>88629.60862998455</v>
       </c>
-      <c r="C106">
+      <c r="E106">
         <v>52500</v>
       </c>
-      <c r="D106">
+      <c r="F106">
         <v>36129.60862998455</v>
       </c>
-      <c r="E106">
+      <c r="G106">
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:5">
+    <row r="107" spans="1:7">
       <c r="A107">
         <v>106</v>
       </c>
       <c r="B107">
+        <v>61244.46043339261</v>
+      </c>
+      <c r="C107">
+        <v>26247.6259000254</v>
+      </c>
+      <c r="D107">
         <v>87492.08633341802</v>
       </c>
-      <c r="C107">
+      <c r="E107">
         <v>53000</v>
       </c>
-      <c r="D107">
+      <c r="F107">
         <v>34492.08633341802</v>
       </c>
-      <c r="E107">
+      <c r="G107">
         <v>9</v>
       </c>
     </row>
-    <row r="108" spans="1:5">
+    <row r="108" spans="1:7">
       <c r="A108">
         <v>107</v>
       </c>
       <c r="B108">
+        <v>57166.37705682755</v>
+      </c>
+      <c r="C108">
+        <v>26760.44898063074</v>
+      </c>
+      <c r="D108">
         <v>83926.82603745829</v>
       </c>
-      <c r="C108">
+      <c r="E108">
         <v>53500</v>
       </c>
-      <c r="D108">
+      <c r="F108">
         <v>30426.82603745829</v>
       </c>
-      <c r="E108">
+      <c r="G108">
         <v>9</v>
       </c>
     </row>
-    <row r="109" spans="1:5">
+    <row r="109" spans="1:7">
       <c r="A109">
         <v>108</v>
       </c>
       <c r="B109">
+        <v>59217.19903808209</v>
+      </c>
+      <c r="C109">
+        <v>27559.84458916818</v>
+      </c>
+      <c r="D109">
         <v>86777.04362725027</v>
       </c>
-      <c r="C109">
+      <c r="E109">
         <v>54000</v>
       </c>
-      <c r="D109">
+      <c r="F109">
         <v>32777.04362725027</v>
       </c>
-      <c r="E109">
+      <c r="G109">
         <v>9</v>
       </c>
     </row>
-    <row r="110" spans="1:5">
+    <row r="110" spans="1:7">
       <c r="A110">
         <v>109</v>
       </c>
       <c r="B110">
+        <v>63627.22618869053</v>
+      </c>
+      <c r="C110">
+        <v>27735.83916204505</v>
+      </c>
+      <c r="D110">
         <v>91363.06535073557</v>
       </c>
-      <c r="C110">
+      <c r="E110">
         <v>54500</v>
       </c>
-      <c r="D110">
+      <c r="F110">
         <v>36863.06535073557</v>
       </c>
-      <c r="E110">
+      <c r="G110">
         <v>10</v>
       </c>
     </row>
-    <row r="111" spans="1:5">
+    <row r="111" spans="1:7">
       <c r="A111">
         <v>110</v>
       </c>
       <c r="B111">
+        <v>66826.37328999204</v>
+      </c>
+      <c r="C111">
+        <v>28095.53151591199</v>
+      </c>
+      <c r="D111">
         <v>94921.90480590402</v>
       </c>
-      <c r="C111">
+      <c r="E111">
         <v>55000</v>
       </c>
-      <c r="D111">
+      <c r="F111">
         <v>39921.90480590402</v>
       </c>
-      <c r="E111">
+      <c r="G111">
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:5">
+    <row r="112" spans="1:7">
       <c r="A112">
         <v>111</v>
       </c>
       <c r="B112">
+        <v>55347.4299277892</v>
+      </c>
+      <c r="C112">
+        <v>26551.3542312415</v>
+      </c>
+      <c r="D112">
         <v>81898.78415903071</v>
       </c>
-      <c r="C112">
+      <c r="E112">
         <v>55500</v>
       </c>
-      <c r="D112">
+      <c r="F112">
         <v>26398.78415903071</v>
       </c>
-      <c r="E112">
+      <c r="G112">
         <v>10</v>
       </c>
     </row>
-    <row r="113" spans="1:5">
+    <row r="113" spans="1:7">
       <c r="A113">
         <v>112</v>
       </c>
       <c r="B113">
+        <v>53134.36581605524</v>
+      </c>
+      <c r="C113">
+        <v>25537.0659101631</v>
+      </c>
+      <c r="D113">
         <v>78671.43172621835</v>
       </c>
-      <c r="C113">
+      <c r="E113">
         <v>56000</v>
       </c>
-      <c r="D113">
+      <c r="F113">
         <v>22671.43172621835</v>
       </c>
-      <c r="E113">
+      <c r="G113">
         <v>10</v>
       </c>
     </row>
-    <row r="114" spans="1:5">
+    <row r="114" spans="1:7">
       <c r="A114">
         <v>113</v>
       </c>
       <c r="B114">
+        <v>55701.65760226624</v>
+      </c>
+      <c r="C114">
+        <v>26551.45668743025</v>
+      </c>
+      <c r="D114">
         <v>82253.11428969649</v>
       </c>
-      <c r="C114">
+      <c r="E114">
         <v>56500</v>
       </c>
-      <c r="D114">
+      <c r="F114">
         <v>25753.11428969649</v>
       </c>
-      <c r="E114">
+      <c r="G114">
         <v>10</v>
       </c>
     </row>
-    <row r="115" spans="1:5">
+    <row r="115" spans="1:7">
       <c r="A115">
         <v>114</v>
       </c>
       <c r="B115">
+        <v>56205.33948613833</v>
+      </c>
+      <c r="C115">
+        <v>26008.31868129725</v>
+      </c>
+      <c r="D115">
         <v>82213.65816743558</v>
       </c>
-      <c r="C115">
+      <c r="E115">
         <v>57000</v>
       </c>
-      <c r="D115">
+      <c r="F115">
         <v>25213.65816743558</v>
       </c>
-      <c r="E115">
+      <c r="G115">
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:5">
+    <row r="116" spans="1:7">
       <c r="A116">
         <v>115</v>
       </c>
       <c r="B116">
+        <v>60047.8014817971</v>
+      </c>
+      <c r="C116">
+        <v>26797.9308268792</v>
+      </c>
+      <c r="D116">
         <v>86845.73230867629</v>
       </c>
-      <c r="C116">
+      <c r="E116">
         <v>57500</v>
       </c>
-      <c r="D116">
+      <c r="F116">
         <v>29345.73230867629</v>
       </c>
-      <c r="E116">
+      <c r="G116">
         <v>10</v>
       </c>
     </row>
-    <row r="117" spans="1:5">
+    <row r="117" spans="1:7">
       <c r="A117">
         <v>116</v>
       </c>
       <c r="B117">
+        <v>64256.20853944617</v>
+      </c>
+      <c r="C117">
+        <v>27284.41850485496</v>
+      </c>
+      <c r="D117">
         <v>91540.62704430113</v>
       </c>
-      <c r="C117">
+      <c r="E117">
         <v>58000</v>
       </c>
-      <c r="D117">
+      <c r="F117">
         <v>33540.62704430113</v>
       </c>
-      <c r="E117">
+      <c r="G117">
         <v>10</v>
       </c>
     </row>
-    <row r="118" spans="1:5">
+    <row r="118" spans="1:7">
       <c r="A118">
         <v>117</v>
       </c>
       <c r="B118">
+        <v>64826.87242791079</v>
+      </c>
+      <c r="C118">
+        <v>27029.65244804898</v>
+      </c>
+      <c r="D118">
         <v>91856.52487595976</v>
       </c>
-      <c r="C118">
+      <c r="E118">
         <v>58500</v>
       </c>
-      <c r="D118">
+      <c r="F118">
         <v>33356.52487595976</v>
       </c>
-      <c r="E118">
+      <c r="G118">
         <v>10</v>
       </c>
     </row>
-    <row r="119" spans="1:5">
+    <row r="119" spans="1:7">
       <c r="A119">
         <v>118</v>
       </c>
       <c r="B119">
+        <v>54276.86797315392</v>
+      </c>
+      <c r="C119">
+        <v>27347.64584947775</v>
+      </c>
+      <c r="D119">
         <v>81624.51382263168</v>
       </c>
-      <c r="C119">
+      <c r="E119">
         <v>59000</v>
       </c>
-      <c r="D119">
+      <c r="F119">
         <v>22624.51382263168</v>
       </c>
-      <c r="E119">
+      <c r="G119">
         <v>10</v>
       </c>
     </row>
-    <row r="120" spans="1:5">
+    <row r="120" spans="1:7">
       <c r="A120">
         <v>119</v>
       </c>
       <c r="B120">
+        <v>63779.74425011565</v>
+      </c>
+      <c r="C120">
+        <v>28032.32672849326</v>
+      </c>
+      <c r="D120">
         <v>91812.0709786089</v>
       </c>
-      <c r="C120">
+      <c r="E120">
         <v>59500</v>
       </c>
-      <c r="D120">
+      <c r="F120">
         <v>32312.0709786089</v>
       </c>
-      <c r="E120">
+      <c r="G120">
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:5">
+    <row r="121" spans="1:7">
       <c r="A121">
         <v>120</v>
       </c>
       <c r="B121">
+        <v>67796.32644436693</v>
+      </c>
+      <c r="C121">
+        <v>28989.55854085735</v>
+      </c>
+      <c r="D121">
         <v>96785.88498522429</v>
       </c>
-      <c r="C121">
+      <c r="E121">
         <v>60000</v>
       </c>
-      <c r="D121">
+      <c r="F121">
         <v>36785.88498522429</v>
       </c>
-      <c r="E121">
+      <c r="G121">
         <v>10</v>
       </c>
     </row>
@@ -4097,15 +4862,58 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="22.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>5</v>
+      <c r="A1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4">
+        <v>96785.88498522429</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>36785.88498522429</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>4.897726957208803</v>
       </c>
     </row>
   </sheetData>

</xml_diff>